<commit_message>
a lot of small changes and quality of life improvements.
</commit_message>
<xml_diff>
--- a/PCB/BOM_PCB.xlsx
+++ b/PCB/BOM_PCB.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="119">
   <si>
     <t>No.</t>
   </si>
@@ -49,7 +49,7 @@
     <t>100nF</t>
   </si>
   <si>
-    <t>C1,C2,C3,C4,C5,C11,C12,C13</t>
+    <t>C1,C6,C7,C12,C13,C14,C17,C18</t>
   </si>
   <si>
     <t>C1206</t>
@@ -73,19 +73,19 @@
     <t>1uF</t>
   </si>
   <si>
-    <t>C6,C7,C8,C9,C10</t>
+    <t>C2,C3,C4,C5,C8,C16</t>
   </si>
   <si>
     <t>CAP-SMD_L3.5-W2.8-R-RD</t>
   </si>
   <si>
-    <t>TAJB105K035RNJ</t>
-  </si>
-  <si>
-    <t>Kyocera AVX</t>
-  </si>
-  <si>
-    <t>C7192</t>
+    <t>293D105X9016A2TE3</t>
+  </si>
+  <si>
+    <t>VISHAY(威世)</t>
+  </si>
+  <si>
+    <t>C162327</t>
   </si>
   <si>
     <t>3</t>
@@ -94,10 +94,10 @@
     <t>1000uF</t>
   </si>
   <si>
-    <t>C14,C15,C16,C17</t>
-  </si>
-  <si>
-    <t>CAP-D10.0×F5.0</t>
+    <t>C9,C10,C11,C15</t>
+  </si>
+  <si>
+    <t>CAP-TH_BD8.0-P3.50-D0.6-FD-H17.0</t>
   </si>
   <si>
     <t>PB25V1000M8X17</t>
@@ -151,7 +151,7 @@
     <t>6</t>
   </si>
   <si>
-    <t>PIC12F1840-E/P</t>
+    <t>PIC12F1840-I/P</t>
   </si>
   <si>
     <t>IC1</t>
@@ -178,13 +178,34 @@
     <t>8</t>
   </si>
   <si>
+    <t>33uH</t>
+  </si>
+  <si>
+    <t>L1</t>
+  </si>
+  <si>
+    <t>IND-TH_BD8.7-P5.0-D0.7_RLB0914</t>
+  </si>
+  <si>
+    <t>RLB0914-330KL</t>
+  </si>
+  <si>
+    <t>BOURNS</t>
+  </si>
+  <si>
+    <t>C1331126</t>
+  </si>
+  <si>
+    <t>9</t>
+  </si>
+  <si>
     <t>SD30CRMA</t>
   </si>
   <si>
     <t>P1</t>
   </si>
   <si>
-    <t>9</t>
+    <t>10</t>
   </si>
   <si>
     <t>AO3416</t>
@@ -202,13 +223,13 @@
     <t>C43307</t>
   </si>
   <si>
-    <t>10</t>
+    <t>11</t>
   </si>
   <si>
     <t>1kΩ</t>
   </si>
   <si>
-    <t>R1,R2,R3,R4,R5,R6,R7,R8,R9,R10,R11,R12,R13,R14,R15,R16,R17,R18,R19,R20,R21,R22,R23,R24,R25,R26</t>
+    <t>R1,R2,R3,R4,R5,R6,R7,R8,R9,R10,R11,R12,R13,R14,R15,R16,R17,R18,R19,R21,R22,R23</t>
   </si>
   <si>
     <t>R1206</t>
@@ -223,25 +244,76 @@
     <t>C2907295</t>
   </si>
   <si>
-    <t>11</t>
+    <t>12</t>
+  </si>
+  <si>
+    <t>4k7</t>
+  </si>
+  <si>
+    <t>R20</t>
+  </si>
+  <si>
+    <t>13</t>
+  </si>
+  <si>
+    <t>LD1086DT33TR</t>
+  </si>
+  <si>
+    <t>U1</t>
+  </si>
+  <si>
+    <t>TO-252-2_L6.5-W6.1-P4.58-LS10.0-TL</t>
+  </si>
+  <si>
+    <t>ST(意法半导体)</t>
+  </si>
+  <si>
+    <t>C12051</t>
+  </si>
+  <si>
+    <t>14</t>
+  </si>
+  <si>
+    <t>TPS63020</t>
+  </si>
+  <si>
+    <t>U2</t>
+  </si>
+  <si>
+    <t>15</t>
   </si>
   <si>
     <t>NRF52840_Nano_v2.0</t>
   </si>
   <si>
-    <t>U1</t>
+    <t>U3</t>
   </si>
   <si>
     <t>NRF52840_NANO_V2,0</t>
   </si>
   <si>
-    <t>12</t>
+    <t>16</t>
+  </si>
+  <si>
+    <t>TSW-102-07-F-S</t>
+  </si>
+  <si>
+    <t>U4,U5,U7,U8,U9,U12</t>
+  </si>
+  <si>
+    <t>HDR-TH_2P-P2.54-V-M-3</t>
+  </si>
+  <si>
+    <t>C3331037</t>
+  </si>
+  <si>
+    <t>17</t>
   </si>
   <si>
     <t>E22P-868M30S</t>
   </si>
   <si>
-    <t>U2</t>
+    <t>U6</t>
   </si>
   <si>
     <t>EBYTE(亿佰特)</t>
@@ -250,64 +322,25 @@
     <t>C51912689</t>
   </si>
   <si>
-    <t>13</t>
+    <t>18</t>
   </si>
   <si>
     <t>DS3231</t>
   </si>
   <si>
-    <t>U3</t>
+    <t>U10</t>
   </si>
   <si>
     <t>IIOTSME</t>
   </si>
   <si>
-    <t>14</t>
-  </si>
-  <si>
-    <t>XL63070</t>
-  </si>
-  <si>
-    <t>U4</t>
-  </si>
-  <si>
-    <t>15</t>
-  </si>
-  <si>
-    <t>TSW-102-07-F-S</t>
-  </si>
-  <si>
-    <t>U5,U6,U8,U12,U13,U14</t>
-  </si>
-  <si>
-    <t>HDR-TH_2P-P2.54-V-M-3</t>
-  </si>
-  <si>
-    <t>C3331037</t>
-  </si>
-  <si>
-    <t>16</t>
-  </si>
-  <si>
-    <t>MCP1727-ADJE/SN</t>
-  </si>
-  <si>
-    <t>U7</t>
-  </si>
-  <si>
-    <t>SOIC-8_L4.9-W3.9-P1.27-LS6.0-BL</t>
-  </si>
-  <si>
-    <t>C635937</t>
-  </si>
-  <si>
-    <t>17</t>
+    <t>19</t>
   </si>
   <si>
     <t>DS18B20+T&amp;R</t>
   </si>
   <si>
-    <t>U9</t>
+    <t>U11</t>
   </si>
   <si>
     <t>TO-92-3_L4.9-W3.7-P2.54-L</t>
@@ -319,40 +352,22 @@
     <t>C880672</t>
   </si>
   <si>
-    <t>18</t>
-  </si>
-  <si>
-    <t>33UH/1A</t>
-  </si>
-  <si>
-    <t>U10</t>
-  </si>
-  <si>
-    <t>IND-TH_BD10.0-P5.00-D0.6</t>
-  </si>
-  <si>
-    <t>33uH/1A</t>
+    <t>20</t>
+  </si>
+  <si>
+    <t>RED</t>
+  </si>
+  <si>
+    <t>U13</t>
+  </si>
+  <si>
+    <t>LED-SMD_CZ1206BH</t>
   </si>
   <si>
     <t>null</t>
   </si>
   <si>
-    <t>C9900019827</t>
-  </si>
-  <si>
-    <t>19</t>
-  </si>
-  <si>
-    <t>CZ1206BH</t>
-  </si>
-  <si>
-    <t>U11</t>
-  </si>
-  <si>
-    <t>LED-SMD_CZ1206BH</t>
-  </si>
-  <si>
-    <t>C9900198175</t>
+    <t>C965812</t>
   </si>
 </sst>
 </file>
@@ -729,7 +744,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J21"/>
+  <dimension ref="A1:J22"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="10" width="20" customWidth="1"/>
@@ -804,7 +819,7 @@
         <v>18</v>
       </c>
       <c r="B3">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C3" t="s">
         <v>19</v>
@@ -1005,77 +1020,77 @@
         <v>56</v>
       </c>
       <c r="E9" t="s">
+        <v>57</v>
+      </c>
+      <c r="F9" t="s">
         <v>55</v>
       </c>
-      <c r="F9" t="s">
-        <v>36</v>
-      </c>
       <c r="G9" t="s">
-        <v>36</v>
+        <v>58</v>
       </c>
       <c r="H9" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="I9" t="s">
-        <v>36</v>
+        <v>60</v>
       </c>
       <c r="J9" t="s">
-        <v>36</v>
+        <v>17</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="B10">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C10" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="D10" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="E10" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="F10" t="s">
         <v>36</v>
       </c>
       <c r="G10" t="s">
-        <v>58</v>
+        <v>36</v>
       </c>
       <c r="H10" t="s">
-        <v>61</v>
+        <v>36</v>
       </c>
       <c r="I10" t="s">
-        <v>62</v>
+        <v>36</v>
       </c>
       <c r="J10" t="s">
-        <v>17</v>
+        <v>36</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B11">
-        <v>26</v>
+        <v>5</v>
       </c>
       <c r="C11" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D11" t="s">
+        <v>66</v>
+      </c>
+      <c r="E11" t="s">
+        <v>67</v>
+      </c>
+      <c r="F11" t="s">
+        <v>36</v>
+      </c>
+      <c r="G11" t="s">
         <v>65</v>
-      </c>
-      <c r="E11" t="s">
-        <v>66</v>
-      </c>
-      <c r="F11" t="s">
-        <v>64</v>
-      </c>
-      <c r="G11" t="s">
-        <v>67</v>
       </c>
       <c r="H11" t="s">
         <v>68</v>
@@ -1092,7 +1107,7 @@
         <v>70</v>
       </c>
       <c r="B12">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="C12" t="s">
         <v>71</v>
@@ -1104,48 +1119,48 @@
         <v>73</v>
       </c>
       <c r="F12" t="s">
-        <v>36</v>
+        <v>71</v>
       </c>
       <c r="G12" t="s">
-        <v>36</v>
+        <v>74</v>
       </c>
       <c r="H12" t="s">
-        <v>36</v>
+        <v>75</v>
       </c>
       <c r="I12" t="s">
-        <v>36</v>
+        <v>76</v>
       </c>
       <c r="J12" t="s">
-        <v>36</v>
+        <v>17</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="B13">
         <v>1</v>
       </c>
       <c r="C13" t="s">
+        <v>78</v>
+      </c>
+      <c r="D13" t="s">
+        <v>79</v>
+      </c>
+      <c r="E13" t="s">
+        <v>73</v>
+      </c>
+      <c r="F13" t="s">
+        <v>71</v>
+      </c>
+      <c r="G13" t="s">
+        <v>74</v>
+      </c>
+      <c r="H13" t="s">
         <v>75</v>
       </c>
-      <c r="D13" t="s">
+      <c r="I13" t="s">
         <v>76</v>
-      </c>
-      <c r="E13" t="s">
-        <v>75</v>
-      </c>
-      <c r="F13" t="s">
-        <v>36</v>
-      </c>
-      <c r="G13" t="s">
-        <v>75</v>
-      </c>
-      <c r="H13" t="s">
-        <v>77</v>
-      </c>
-      <c r="I13" t="s">
-        <v>78</v>
       </c>
       <c r="J13" t="s">
         <v>17</v>
@@ -1153,57 +1168,57 @@
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B14">
         <v>1</v>
       </c>
       <c r="C14" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D14" t="s">
+        <v>82</v>
+      </c>
+      <c r="E14" t="s">
+        <v>83</v>
+      </c>
+      <c r="F14" t="s">
+        <v>36</v>
+      </c>
+      <c r="G14" t="s">
         <v>81</v>
       </c>
-      <c r="E14" t="s">
-        <v>80</v>
-      </c>
-      <c r="F14" t="s">
-        <v>36</v>
-      </c>
-      <c r="G14" t="s">
-        <v>80</v>
-      </c>
       <c r="H14" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="I14" t="s">
-        <v>36</v>
+        <v>85</v>
       </c>
       <c r="J14" t="s">
-        <v>82</v>
+        <v>17</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="B15">
         <v>1</v>
       </c>
       <c r="C15" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="D15" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="E15" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="F15" t="s">
         <v>36</v>
       </c>
       <c r="G15" t="s">
-        <v>36</v>
+        <v>87</v>
       </c>
       <c r="H15" t="s">
         <v>36</v>
@@ -1217,63 +1232,63 @@
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="B16">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C16" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="D16" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="E16" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="F16" t="s">
         <v>36</v>
       </c>
       <c r="G16" t="s">
-        <v>87</v>
+        <v>36</v>
       </c>
       <c r="H16" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="I16" t="s">
-        <v>90</v>
+        <v>36</v>
       </c>
       <c r="J16" t="s">
-        <v>17</v>
+        <v>36</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B17">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C17" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D17" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="E17" t="s">
+        <v>96</v>
+      </c>
+      <c r="F17" t="s">
+        <v>36</v>
+      </c>
+      <c r="G17" t="s">
         <v>94</v>
       </c>
-      <c r="F17" t="s">
-        <v>36</v>
-      </c>
-      <c r="G17" t="s">
-        <v>92</v>
-      </c>
       <c r="H17" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="I17" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="J17" t="s">
         <v>17</v>
@@ -1281,16 +1296,16 @@
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B18">
         <v>1</v>
       </c>
       <c r="C18" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="D18" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="E18" t="s">
         <v>99</v>
@@ -1299,13 +1314,13 @@
         <v>36</v>
       </c>
       <c r="G18" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="H18" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="I18" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="J18" t="s">
         <v>17</v>
@@ -1313,70 +1328,102 @@
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B19">
         <v>1</v>
       </c>
       <c r="C19" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D19" t="s">
+        <v>105</v>
+      </c>
+      <c r="E19" t="s">
         <v>104</v>
       </c>
-      <c r="E19" t="s">
-        <v>105</v>
-      </c>
       <c r="F19" t="s">
         <v>36</v>
       </c>
       <c r="G19" t="s">
+        <v>104</v>
+      </c>
+      <c r="H19" t="s">
         <v>106</v>
       </c>
-      <c r="H19" t="s">
-        <v>107</v>
-      </c>
       <c r="I19" t="s">
-        <v>108</v>
+        <v>36</v>
       </c>
       <c r="J19" t="s">
-        <v>17</v>
+        <v>106</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="B20">
         <v>1</v>
       </c>
       <c r="C20" t="s">
+        <v>108</v>
+      </c>
+      <c r="D20" t="s">
+        <v>109</v>
+      </c>
+      <c r="E20" t="s">
         <v>110</v>
       </c>
-      <c r="D20" t="s">
+      <c r="F20" t="s">
+        <v>36</v>
+      </c>
+      <c r="G20" t="s">
+        <v>108</v>
+      </c>
+      <c r="H20" t="s">
         <v>111</v>
       </c>
-      <c r="E20" t="s">
+      <c r="I20" t="s">
         <v>112</v>
-      </c>
-      <c r="F20" t="s">
-        <v>36</v>
-      </c>
-      <c r="G20" t="s">
-        <v>110</v>
-      </c>
-      <c r="H20" t="s">
-        <v>107</v>
-      </c>
-      <c r="I20" t="s">
-        <v>113</v>
       </c>
       <c r="J20" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>113</v>
+      </c>
+      <c r="B21">
+        <v>1</v>
+      </c>
+      <c r="C21" t="s">
+        <v>114</v>
+      </c>
+      <c r="D21" t="s">
+        <v>115</v>
+      </c>
+      <c r="E21" t="s">
+        <v>116</v>
+      </c>
+      <c r="F21" t="s">
+        <v>36</v>
+      </c>
+      <c r="G21" t="s">
+        <v>36</v>
+      </c>
+      <c r="H21" t="s">
+        <v>117</v>
+      </c>
+      <c r="I21" t="s">
+        <v>118</v>
+      </c>
+      <c r="J21" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
         <v>36</v>
       </c>
     </row>

</xml_diff>